<commit_message>
added import options and also bulk owner assignement
</commit_message>
<xml_diff>
--- a/odoo_nhs_dspt/static/import_templates/dspt_assertions_import_template.xlsx
+++ b/odoo_nhs_dspt/static/import_templates/dspt_assertions_import_template.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -416,22 +417,22 @@
   <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>standard_id/edition_id/year</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>standard_id/code</t>
+          <t>standard_id/id</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -450,8 +451,201 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
-    <row r="3"/>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>__import__.dspt_assertion_demo_1_2</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>odoo_nhs_dspt.std_1_personal_data</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Sample assertion — Personal data is only retained as long as necessary</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>__import__.dspt_assertion_demo_2_2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>odoo_nhs_dspt.std_2_staff_responsibilities</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Sample assertion — Staff sign an annual confidentiality declaration</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>HOW THE 'id' COLUMNS WORK</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Odoo's generic import can only match an EXISTING related record via its External ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>(the 'xxx_id/id' columns below) or its database id — it cannot create a missing parent</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>record on the fly from a name/code/reference value. The sample rows below reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>the External IDs shipped with this module's seed data, so they import cleanly as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>'id' (first column): assigns a NEW External ID to the row you are creating. Do NOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>prefix it with 'odoo_nhs_dspt.' (or any other installed module's name) — Odoo will</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>refuse the import, because a record filed under another module's prefix gets deleted</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>the next time that module is upgraded. Use the '__import__.' prefix instead (Odoo's</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>own recommended convention for imported data), e.g. '__import__.my_new_standard_2027'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>To find the External ID of a record you created yourself (for the 'xxx_id/id' lookup</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>columns): enable Developer Mode (Settings &gt; General Settings &gt; Developer Tools), open</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>the record, then Actions (gear icon) &gt; View Metadata.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>THIS SHEET: creates 2 new Assertions under the seed Standards 1 (Personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Confidential Data) and 2 (Staff Responsibilities) — try importing it as-is first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>reference must be unique within the edition (e.g. '1.1' already exists and would</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>raise a validation error if reused; '1.2' is new).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>